<commit_message>
Bug fix for unhandled ArrowStringError when using newer versions of Pandas
</commit_message>
<xml_diff>
--- a/example_data/metadata.xlsx
+++ b/example_data/metadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Pycharm Projects\claude_pythomics\test_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/max/Documents/GitHub/ClockWork/example_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CAC0D7D-714A-49A3-82ED-1E9369E20432}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="885" windowWidth="29040" windowHeight="15720" xr2:uid="{C1332F9D-CA6F-40F0-B8AB-D048349F05D6}"/>
+    <workbookView xWindow="12520" yWindow="960" windowWidth="28800" windowHeight="16300" xr2:uid="{C1332F9D-CA6F-40F0-B8AB-D048349F05D6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -573,14 +573,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
@@ -958,17 +953,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24F859B2-972D-48E6-B53C-9868CC37BA1F}">
   <dimension ref="A1:F8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.1640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="7.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="31.6640625" customWidth="1"/>
     <col min="5" max="5" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -988,7 +983,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
@@ -1008,7 +1003,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -1018,7 +1013,7 @@
       <c r="C3">
         <v>18</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E3" t="s">
@@ -1028,7 +1023,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
@@ -1038,7 +1033,7 @@
       <c r="C4">
         <v>19</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="2" t="s">
         <v>12</v>
       </c>
       <c r="E4" t="s">
@@ -1048,7 +1043,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
@@ -1058,7 +1053,7 @@
       <c r="C5">
         <v>20</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="2" t="s">
         <v>13</v>
       </c>
       <c r="E5" t="s">
@@ -1068,7 +1063,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
@@ -1078,7 +1073,7 @@
       <c r="C6">
         <v>21</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E6" t="s">
@@ -1088,7 +1083,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
@@ -1098,7 +1093,7 @@
       <c r="C7">
         <v>22</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="2" t="s">
         <v>15</v>
       </c>
       <c r="E7" t="s">
@@ -1108,7 +1103,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
     </row>

</xml_diff>